<commit_message>
웹앱 업데이트 2026-10-16 01:03
</commit_message>
<xml_diff>
--- a/tripflip-template.xlsx
+++ b/tripflip-template.xlsx
@@ -207,40 +207,45 @@
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>앱이 이 글자로 위치를 찾아요. 영어 이름이 가장 정확해요</t>
+        <t>구글맵에 등록된 공식 영어 이름. 주소와 함께 위치를 찾을 때 써요</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
+        <t>실제 주소를 영어로, "번지 도로명, 동네, 도시 우편번호, 국가" 순서로 쉼표로 나눠서 (장소 이름은 빼고). 앱이 이 주소로 위치를 찾아요</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
         <t>머무는 시간. 60, 1:30, 1시간 30분 모두 가능</t>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
+    <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <t>그 장소까지 가는 방법: 도보 / 대중교통 / 차량 / 자전거</t>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <t>상세 페이지에 보여요</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <t>"a. 카페  b. 서점" 처럼 적으면 앱에서 누를 수 있는 버튼이 돼요</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+    <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <t>예약 번호, 할 일 등</t>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
+    <comment ref="K1" authorId="0" shapeId="0">
       <text>
         <t>선택. 적으면 검색보다 정확 (구글맵에서 장소를 길게 누르면 나오는 숫자)</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
+    <comment ref="L1" authorId="0" shapeId="0">
       <text>
         <t>선택</t>
       </text>
@@ -538,20 +543,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:L10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -572,40 +578,45 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>주소(검색어)</t>
+          <t>영문 이름</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
+          <t>주소</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
           <t>체류(분)</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>이동수단</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>설명</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>주변 추천</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>메모</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>위도</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>경도</t>
         </is>
@@ -629,20 +640,25 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Hotel Gracery Shinjuku Tokyo</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="n"/>
+          <t>Hotel Gracery Shinjuku</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>1-19-1 Kabukicho, Shinjuku City, Tokyo 160-8466, Japan</t>
+        </is>
+      </c>
       <c r="F2" s="4" t="n"/>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>첫날 출발</t>
         </is>
       </c>
-      <c r="H2" s="5" t="n"/>
       <c r="I2" s="5" t="n"/>
-      <c r="J2" s="4" t="n"/>
+      <c r="J2" s="5" t="n"/>
       <c r="K2" s="4" t="n"/>
+      <c r="L2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n"/>
@@ -654,30 +670,35 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Meiji Jingu Shrine Tokyo</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="n">
+          <t>Meiji Jingu</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>1-1 Yoyogikamizonocho, Shibuya City, Tokyo 151-8557, Japan</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>대중교통</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>도심 속 큰 숲길 산책</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>a. 요요기 공원  b. 하라주쿠역</t>
         </is>
       </c>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="4" t="n"/>
+      <c r="J3" s="5" t="n"/>
       <c r="K3" s="4" t="n"/>
+      <c r="L3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n"/>
@@ -693,26 +714,31 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Shibuya Station Tokyo</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="n">
+          <t>Shibuya Station</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>2-24 Shibuya, Shibuya City, Tokyo 150-0002, Japan</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>도보</t>
         </is>
       </c>
-      <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="5" t="n"/>
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>점심 예약 12:30 (예약번호 1234)</t>
         </is>
       </c>
-      <c r="J4" s="4" t="n"/>
       <c r="K4" s="4" t="n"/>
+      <c r="L4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n"/>
@@ -724,30 +750,35 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Shibuya Sky Tokyo</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="n">
+          <t>SHIBUYA SKY</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>2-24-12 Shibuya, Shibuya City, Tokyo 150-6145, Japan</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
         <v>90</v>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>도보</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>전망대. 해 질 녘이 가장 예뻐요</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>a. 스크램블 교차로  b. 미야시타 파크</t>
         </is>
       </c>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="4" t="n"/>
+      <c r="J5" s="5" t="n"/>
       <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -759,24 +790,29 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Hotel Gracery Shinjuku Tokyo</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="inlineStr">
+          <t>Hotel Gracery Shinjuku</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>1-19-1 Kabukicho, Shinjuku City, Tokyo 160-8466, Japan</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>대중교통</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>숙소 복귀</t>
         </is>
       </c>
-      <c r="H6" s="5" t="n"/>
       <c r="I6" s="5" t="n"/>
-      <c r="J6" s="4" t="n"/>
+      <c r="J6" s="5" t="n"/>
       <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -796,16 +832,21 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Hotel Gracery Shinjuku Tokyo</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="n"/>
+          <t>Hotel Gracery Shinjuku</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>1-19-1 Kabukicho, Shinjuku City, Tokyo 160-8466, Japan</t>
+        </is>
+      </c>
       <c r="F7" s="4" t="n"/>
-      <c r="G7" s="5" t="n"/>
+      <c r="G7" s="4" t="n"/>
       <c r="H7" s="5" t="n"/>
       <c r="I7" s="5" t="n"/>
-      <c r="J7" s="4" t="n"/>
+      <c r="J7" s="5" t="n"/>
       <c r="K7" s="4" t="n"/>
+      <c r="L7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>
@@ -817,26 +858,31 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Sensoji Temple Tokyo</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="n">
+          <t>Senso-ji</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>2-3-1 Asakusa, Taito City, Tokyo 111-0032, Japan</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
         <v>90</v>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>대중교통</t>
         </is>
       </c>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>a. 나카미세 거리  b. 아사쿠사 문화관광센터</t>
         </is>
       </c>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="4" t="n"/>
+      <c r="J8" s="5" t="n"/>
       <c r="K8" s="4" t="n"/>
+      <c r="L8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n"/>
@@ -855,23 +901,28 @@
           <t>Tokyo Skytree</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>1-1-2 Oshiage, Sumida City, Tokyo 131-0045, Japan</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
         <v>90</v>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>대중교통</t>
         </is>
       </c>
-      <c r="G9" s="5" t="n"/>
       <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I9" s="5" t="n"/>
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>전망대 14:00 입장권</t>
         </is>
       </c>
-      <c r="J9" s="4" t="n"/>
       <c r="K9" s="4" t="n"/>
+      <c r="L9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
@@ -883,24 +934,29 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Hotel Gracery Shinjuku Tokyo</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="inlineStr">
+          <t>Hotel Gracery Shinjuku</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>1-19-1 Kabukicho, Shinjuku City, Tokyo 160-8466, Japan</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>대중교통</t>
         </is>
       </c>
-      <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="n"/>
       <c r="I10" s="5" t="n"/>
-      <c r="J10" s="4" t="n"/>
+      <c r="J10" s="5" t="n"/>
       <c r="K10" s="4" t="n"/>
+      <c r="L10" s="4" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"도보,대중교통,차량,자전거"</formula1>
     </dataValidation>
   </dataValidations>
@@ -915,8 +971,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:A15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
@@ -962,50 +1018,57 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>5. 주소(검색어): 앱이 이 글자로 위치를 찾아요. "Meiji Jingu Shrine Tokyo"처럼 영어 이름 + 도시가 가장 정확해요.</t>
+          <t>5. 영문 이름 + 주소: 앱이 이 두 칸으로 지도 위치를 찾아요. 주소는 영어로 "번지 도로명, 동네, 도시 우편번호, 국가"처럼 쉼표로 나눠 적고, 장소 이름은 넣지 마세요.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>6. 체류(분): 그곳에서 머무는 시간. 비우면 다음 장소 시간에 맞춰 계산해요.</t>
+          <t xml:space="preserve">   ChatGPT·Claude·Gemini에게 맡기면 정확한 영문 이름과 주소를 찾아 채워 줘요 (앱의 "일정 양식 · AI로 만들기" 문구를 쓰세요).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>7. 이동수단: 그 장소까지 가는 방법. 칸을 누르면 도보/대중교통/차량/자전거 중에서 고를 수 있어요.</t>
+          <t>6. 체류(분): 그곳에서 머무는 시간. 비우면 다음 장소 시간에 맞춰 계산해요.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>8. 하루 마지막은 숙소로 돌아오는 줄을 넣으면 좋아요. 빠뜨리면 앱이 숙소 복귀를 자동으로 붙여요.</t>
+          <t>7. 이동수단: 그 장소까지 가는 방법. 칸을 누르면 도보/대중교통/차량/자전거 중에서 고를 수 있어요.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
+          <t>8. 하루 마지막은 숙소로 돌아오는 줄을 넣으면 좋아요. 빠뜨리면 앱이 숙소 복귀를 자동으로 붙여요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
           <t>9. 다 적었으면 저장 → 휴대폰으로 보내기 → 트립플립 ⚙️ 설정 → "📂 엑셀/CSV 일정 불러오기".</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>※ 열 순서는 바꿔도 되고, 필요 없는 열은 지워도 돼요. 머리글 이름만 그대로 두세요.</t>
-        </is>
-      </c>
+      <c r="A13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>※ 열 순서는 바꿔도 되고, 필요 없는 열은 지워도 돼요. 머리글 이름만 그대로 두세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>※ 날짜별로 시트를 나눠도 돼요. 이때는 시트 이름을 "11.03" 처럼 날짜로 하거나, 표 위에 "11월 3일" 제목을 적어 주세요.</t>
         </is>

</xml_diff>

<commit_message>
웹앱 업데이트 2026-10-29 19:27
</commit_message>
<xml_diff>
--- a/tripflip-template.xlsx
+++ b/tripflip-template.xlsx
@@ -187,7 +187,7 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>트립플립</author>
+    <author>버블트립</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
@@ -980,7 +980,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>트립플립 일정 양식 사용법</t>
+          <t>버블트립 일정 양식 사용법</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>9. 다 적었으면 저장 → 휴대폰으로 보내기 → 트립플립 ⚙️ 설정 → "📂 엑셀/CSV 일정 불러오기".</t>
+          <t>9. 다 적었으면 저장 → 휴대폰으로 보내기 → 버블트립 ⚙️ 설정 → "📂 엑셀/CSV 일정 불러오기".</t>
         </is>
       </c>
     </row>

</xml_diff>